<commit_message>
Workbook update 2026-09-22 18:01: expense rows +1, bank rows +0, review 0, superseded 0
</commit_message>
<xml_diff>
--- a/output/kosibah_import.xlsx
+++ b/output/kosibah_import.xlsx
@@ -176,9 +176,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="KosibahImport" displayName="KosibahImport" ref="B3:P42" headerRowCount="1">
-  <autoFilter ref="B3:P42"/>
-  <tableColumns count="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="KosibahImport" displayName="KosibahImport" ref="B3:Q43" headerRowCount="1">
+  <autoFilter ref="B3:Q43"/>
+  <tableColumns count="16">
     <tableColumn id="2" name="Date"/>
     <tableColumn id="3" name="Company"/>
     <tableColumn id="4" name="Category"/>
@@ -194,6 +194,7 @@
     <tableColumn id="14" name="Processed on"/>
     <tableColumn id="15" name="Status"/>
     <tableColumn id="16" name="Bank ref"/>
+    <tableColumn id="17" name="Copied to master"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
@@ -508,7 +509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:P43"/>
+  <dimension ref="B1:Q44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -526,6 +527,7 @@
     <col width="18" customWidth="1" min="14" max="14"/>
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="24" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -611,6 +613,11 @@
           <t>Bank ref</t>
         </is>
       </c>
+      <c r="Q3" s="1" t="inlineStr">
+        <is>
+          <t>Copied to master</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="B4" s="2" t="n">
@@ -669,6 +676,7 @@
         </is>
       </c>
       <c r="P4" s="3" t="inlineStr"/>
+      <c r="Q4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="B5" s="7" t="n">
@@ -727,6 +735,7 @@
         </is>
       </c>
       <c r="P5" s="8" t="inlineStr"/>
+      <c r="Q5" s="8" t="n"/>
     </row>
     <row r="6">
       <c r="B6" s="2" t="n">
@@ -785,6 +794,7 @@
         </is>
       </c>
       <c r="P6" s="3" t="inlineStr"/>
+      <c r="Q6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="B7" s="2" t="n">
@@ -843,6 +853,7 @@
         </is>
       </c>
       <c r="P7" s="3" t="inlineStr"/>
+      <c r="Q7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="B8" s="2" t="n">
@@ -901,6 +912,7 @@
         </is>
       </c>
       <c r="P8" s="3" t="inlineStr"/>
+      <c r="Q8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="B9" s="7" t="n">
@@ -963,6 +975,7 @@
           <t>bank/2026 - JUNE JULY AUGUST CAPITAL ONE TRANSACTIONS Yemi Osunkoya.csv#26</t>
         </is>
       </c>
+      <c r="Q9" s="8" t="n"/>
     </row>
     <row r="10">
       <c r="B10" s="2" t="n">
@@ -1025,6 +1038,7 @@
           <t>bank/2026 - JUNE JULY AUGUST CAPITAL ONE TRANSACTIONS Yemi Osunkoya.csv#24</t>
         </is>
       </c>
+      <c r="Q10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="B11" s="2" t="n">
@@ -1087,6 +1101,7 @@
           <t>bank/2026 - JUNE JULY AUGUST CAPITAL ONE TRANSACTIONS Yemi Osunkoya.csv#25</t>
         </is>
       </c>
+      <c r="Q11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="B12" s="2" t="n">
@@ -1149,6 +1164,7 @@
           <t>bank/2026 - JUNE JULY AUGUST CAPITAL ONE TRANSACTIONS Yemi Osunkoya.csv#20</t>
         </is>
       </c>
+      <c r="Q12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="B13" s="2" t="n">
@@ -1211,6 +1227,7 @@
           <t>bank/2026 - JUNE JULY AUGUST CAPITAL ONE TRANSACTIONS Yemi Osunkoya.csv#15</t>
         </is>
       </c>
+      <c r="Q13" s="3" t="n"/>
     </row>
     <row r="14">
       <c r="B14" s="2" t="n">
@@ -1273,6 +1290,7 @@
           <t>bank/2026 - JUNE JULY AUGUST CAPITAL ONE TRANSACTIONS Yemi Osunkoya.csv#19</t>
         </is>
       </c>
+      <c r="Q14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="B15" s="2" t="n">
@@ -1335,6 +1353,7 @@
           <t>bank/2026 - JUNE JULY AUGUST CAPITAL ONE TRANSACTIONS Yemi Osunkoya.csv#18</t>
         </is>
       </c>
+      <c r="Q15" s="3" t="n"/>
     </row>
     <row r="16">
       <c r="B16" s="2" t="n">
@@ -1397,6 +1416,7 @@
           <t>bank/2026 - JUNE JULY AUGUST CAPITAL ONE TRANSACTIONS Yemi Osunkoya.csv#17</t>
         </is>
       </c>
+      <c r="Q16" s="3" t="n"/>
     </row>
     <row r="17">
       <c r="B17" s="2" t="n">
@@ -1459,6 +1479,7 @@
           <t>bank/2026 - JUNE JULY AUGUST CAPITAL ONE TRANSACTIONS Yemi Osunkoya.csv#16</t>
         </is>
       </c>
+      <c r="Q17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="B18" s="2" t="n">
@@ -1521,6 +1542,7 @@
           <t>bank/2026 - JUNE JULY AUGUST CAPITAL ONE TRANSACTIONS Yemi Osunkoya.csv#14</t>
         </is>
       </c>
+      <c r="Q18" s="3" t="n"/>
     </row>
     <row r="19">
       <c r="B19" s="2" t="n">
@@ -1583,6 +1605,7 @@
           <t>bank/2026 - JUNE JULY AUGUST CAPITAL ONE TRANSACTIONS Yemi Osunkoya.csv#13</t>
         </is>
       </c>
+      <c r="Q19" s="3" t="n"/>
     </row>
     <row r="20">
       <c r="B20" s="2" t="n">
@@ -1645,6 +1668,7 @@
           <t>bank/2026 - JUNE JULY AUGUST CAPITAL ONE TRANSACTIONS Yemi Osunkoya.csv#12</t>
         </is>
       </c>
+      <c r="Q20" s="3" t="n"/>
     </row>
     <row r="21">
       <c r="B21" s="2" t="n">
@@ -1703,6 +1727,7 @@
         </is>
       </c>
       <c r="P21" s="3" t="inlineStr"/>
+      <c r="Q21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="B22" s="2" t="n">
@@ -1765,6 +1790,7 @@
           <t>bank/2026 - JUNE JULY AUGUST CAPITAL ONE TRANSACTIONS Yemi Osunkoya.csv#9</t>
         </is>
       </c>
+      <c r="Q22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="B23" s="2" t="n">
@@ -1823,6 +1849,7 @@
         </is>
       </c>
       <c r="P23" s="3" t="inlineStr"/>
+      <c r="Q23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="B24" s="2" t="n">
@@ -1885,6 +1912,7 @@
           <t>bank/2026 - JUNE JULY AUGUST CAPITAL ONE TRANSACTIONS Yemi Osunkoya.csv#7</t>
         </is>
       </c>
+      <c r="Q24" s="3" t="n"/>
     </row>
     <row r="25">
       <c r="B25" s="2" t="n">
@@ -1943,6 +1971,7 @@
         </is>
       </c>
       <c r="P25" s="3" t="inlineStr"/>
+      <c r="Q25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="B26" s="2" t="n">
@@ -2001,6 +2030,7 @@
         </is>
       </c>
       <c r="P26" s="3" t="inlineStr"/>
+      <c r="Q26" s="3" t="n"/>
     </row>
     <row r="27">
       <c r="B27" s="2" t="n">
@@ -2059,6 +2089,7 @@
         </is>
       </c>
       <c r="P27" s="3" t="inlineStr"/>
+      <c r="Q27" s="3" t="n"/>
     </row>
     <row r="28">
       <c r="B28" s="2" t="n">
@@ -2121,6 +2152,7 @@
           <t>bank/2026 - JUNE JULY AUGUST CAPITAL ONE TRANSACTIONS Yemi Osunkoya.csv#2</t>
         </is>
       </c>
+      <c r="Q28" s="3" t="n"/>
     </row>
     <row r="29">
       <c r="B29" s="2" t="n">
@@ -2183,6 +2215,7 @@
           <t>bank/2026 - JUNE JULY AUGUST CAPITAL ONE TRANSACTIONS Yemi Osunkoya.csv#1</t>
         </is>
       </c>
+      <c r="Q29" s="3" t="n"/>
     </row>
     <row r="30">
       <c r="B30" s="7" t="n">
@@ -2245,6 +2278,7 @@
           <t>bank/2026 - JUNE JULY AUGUST CAPITAL ONE TRANSACTIONS Yemi Osunkoya.csv#21</t>
         </is>
       </c>
+      <c r="Q30" s="8" t="n"/>
     </row>
     <row r="31">
       <c r="B31" s="2" t="n">
@@ -2303,6 +2337,7 @@
         </is>
       </c>
       <c r="P31" s="3" t="inlineStr"/>
+      <c r="Q31" s="3" t="n"/>
     </row>
     <row r="32">
       <c r="B32" s="2" t="n">
@@ -2361,6 +2396,7 @@
         </is>
       </c>
       <c r="P32" s="3" t="inlineStr"/>
+      <c r="Q32" s="3" t="n"/>
     </row>
     <row r="33">
       <c r="B33" s="2" t="n">
@@ -2419,6 +2455,7 @@
         </is>
       </c>
       <c r="P33" s="3" t="inlineStr"/>
+      <c r="Q33" s="3" t="n"/>
     </row>
     <row r="34">
       <c r="B34" s="2" t="n">
@@ -2477,6 +2514,7 @@
         </is>
       </c>
       <c r="P34" s="3" t="inlineStr"/>
+      <c r="Q34" s="3" t="n"/>
     </row>
     <row r="35">
       <c r="B35" s="2" t="n">
@@ -2535,6 +2573,7 @@
         </is>
       </c>
       <c r="P35" s="3" t="inlineStr"/>
+      <c r="Q35" s="3" t="n"/>
     </row>
     <row r="36">
       <c r="B36" s="2" t="n">
@@ -2593,6 +2632,7 @@
         </is>
       </c>
       <c r="P36" s="3" t="inlineStr"/>
+      <c r="Q36" s="3" t="n"/>
     </row>
     <row r="37">
       <c r="B37" s="2" t="n">
@@ -2651,6 +2691,7 @@
         </is>
       </c>
       <c r="P37" s="3" t="inlineStr"/>
+      <c r="Q37" s="3" t="n"/>
     </row>
     <row r="38">
       <c r="B38" s="2" t="n">
@@ -2709,6 +2750,7 @@
         </is>
       </c>
       <c r="P38" s="3" t="inlineStr"/>
+      <c r="Q38" s="3" t="n"/>
     </row>
     <row r="39">
       <c r="B39" s="2" t="n">
@@ -2767,6 +2809,7 @@
         </is>
       </c>
       <c r="P39" s="3" t="inlineStr"/>
+      <c r="Q39" s="3" t="n"/>
     </row>
     <row r="40">
       <c r="B40" s="2" t="n">
@@ -2817,7 +2860,7 @@
         </is>
       </c>
       <c r="N40" s="24" t="n">
-        <v>46286.86163054546</v>
+        <v>46286.86163054398</v>
       </c>
       <c r="O40" s="3" t="inlineStr">
         <is>
@@ -2825,6 +2868,7 @@
         </is>
       </c>
       <c r="P40" s="3" t="inlineStr"/>
+      <c r="Q40" s="3" t="n"/>
     </row>
     <row r="41">
       <c r="B41" s="2" t="n">
@@ -2875,7 +2919,7 @@
         </is>
       </c>
       <c r="N41" s="24" t="n">
-        <v>46286.86163054546</v>
+        <v>46286.86163054398</v>
       </c>
       <c r="O41" s="3" t="inlineStr">
         <is>
@@ -2883,6 +2927,7 @@
         </is>
       </c>
       <c r="P41" s="3" t="inlineStr"/>
+      <c r="Q41" s="3" t="n"/>
     </row>
     <row r="42">
       <c r="B42" s="2" t="n">
@@ -2933,7 +2978,7 @@
         </is>
       </c>
       <c r="N42" s="24" t="n">
-        <v>46286.86163054546</v>
+        <v>46286.86163054398</v>
       </c>
       <c r="O42" s="3" t="inlineStr">
         <is>
@@ -2941,23 +2986,83 @@
         </is>
       </c>
       <c r="P42" s="3" t="inlineStr"/>
+      <c r="Q42" s="3" t="n"/>
     </row>
     <row r="43">
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Preview Textiles LLC</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>Fabric</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="n">
+        <v>148</v>
+      </c>
+      <c r="F43" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="4" t="n">
+        <v>148</v>
+      </c>
+      <c r="H43" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>Discover</t>
+        </is>
+      </c>
+      <c r="J43" s="3">
+        <f>IF(ROUND(E43+F43,2)=ROUND(G43,2),"ok","!!!!")</f>
+        <v/>
+      </c>
+      <c r="K43" s="3" t="inlineStr">
+        <is>
+          <t>Description column text overlaps with a stamped/handwritten box (address block), partially obscuring item description and other notations (e.g. '3PM', 'WAITING'); No sales tax line shown on receipt; Card terminal printout (Discover chip transaction, CapitalOne Debit) embedded alongside invoice fields</t>
+        </is>
+      </c>
+      <c r="L43" s="3" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M43" s="3" t="inlineStr">
+        <is>
+          <t>expenses/2026-09-22 Preview Textiles LLC.pdf</t>
+        </is>
+      </c>
+      <c r="N43" s="24" t="n">
+        <v>46287.75077233725</v>
+      </c>
+      <c r="O43" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="P43" s="3" t="inlineStr"/>
+      <c r="Q43" s="3" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="B44" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="E43" s="12">
-        <f>SUBTOTAL(109,E4:E42)</f>
+      <c r="E44" s="12">
+        <f>SUBTOTAL(109,E4:E43)</f>
         <v/>
       </c>
-      <c r="F43" s="12">
-        <f>SUBTOTAL(109,F4:F42)</f>
+      <c r="F44" s="12">
+        <f>SUBTOTAL(109,F4:F43)</f>
         <v/>
       </c>
-      <c r="G43" s="12">
-        <f>SUBTOTAL(109,G4:G42)</f>
+      <c r="G44" s="12">
+        <f>SUBTOTAL(109,G4:G43)</f>
         <v/>
       </c>
     </row>

</xml_diff>